<commit_message>
Bring input_datasets.xlsx and its generator into agreement (0.15, Jan-Mar)
The committed workbook (2026-08) and paper/tables/build_input_datasets_xlsx.py
disagreed. Settled against friction_config.py, confirmed by the owner:

- River ice is thresholded at RIVER_ICE_THRESHOLD = 0.15. The generator still
  said 0.50 with no source; it now carries the workbook's 0.15 description and
  the Brown et al. 2026 source, citing the pipeline at its current path
  (friction_preprocessing/, not the pre-merge gee_scripts/).
- The ice-road season is ICE_ROAD_SEASON_MONTHS = Jan-Mar. The workbook said
  Jan-Apr; regenerated from the generator, which already said Jan-Mar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YCXn1oLPELcXhFBK1cZkc8
</commit_message>
<xml_diff>
--- a/outputs/tables/input_datasets.xlsx
+++ b/outputs/tables/input_datasets.xlsx
@@ -472,7 +472,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -570,7 +569,7 @@
       <c r="C9" s="5" t="inlineStr"/>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Overland ice-road centerlines (packed-snow tundra routes) burned into the overland network during the Jan-Apr season.</t>
+          <t>Overland ice-road centerlines (packed-snow tundra routes) burned into the overland network during the Jan-Mar season.</t>
         </is>
       </c>
     </row>
@@ -610,7 +609,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -671,7 +669,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Brown et al. 2026 (DOI 10.18739/A2SB3X15X), processed by gee_scripts/river_ice_full_pipeline.py</t>
+          <t>Brown et al. 2026 (DOI 10.18739/A2SB3X15X), processed by friction_preprocessing/river_ice_full_pipeline.py</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">

</xml_diff>